<commit_message>
Update modules for version 2.0.0
</commit_message>
<xml_diff>
--- a/1_Stoichiometry_generator/Results.xlsx
+++ b/1_Stoichiometry_generator/Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitry.bublikov\Desktop\Desktop\nacl\NaCl-superstructure-simulator\1_Stoichiometry_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC19614-F0D7-44F4-8DD6-13E63590BFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84B0637-F6A9-4D0B-BAD7-7724A9E919D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -443,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -492,6 +492,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,10 +843,10 @@
       <c r="B4" s="7">
         <v>41515514</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="18">
         <v>2.6620370370370372E-4</v>
       </c>
-      <c r="D4" s="30">
+      <c r="D4" s="36">
         <v>393037764859</v>
       </c>
       <c r="E4" s="30">
@@ -1323,7 +1324,7 @@
         <v>71</v>
       </c>
       <c r="B27" s="7">
-        <v>91979</v>
+        <v>91980</v>
       </c>
       <c r="C27" s="12">
         <v>1.1574074074074073E-5</v>
@@ -1333,7 +1334,7 @@
       </c>
       <c r="E27" s="27">
         <f t="shared" si="0"/>
-        <v>66842220</v>
+        <v>66842219</v>
       </c>
       <c r="F27" s="18">
         <v>7.3263888888888892E-3</v>
@@ -1344,7 +1345,7 @@
         <v>61</v>
       </c>
       <c r="B28" s="7">
-        <v>74493</v>
+        <v>74494</v>
       </c>
       <c r="C28" s="12">
         <v>1.1574074074074073E-5</v>
@@ -1354,7 +1355,7 @@
       </c>
       <c r="E28" s="27">
         <f t="shared" si="0"/>
-        <v>13708673</v>
+        <v>13708672</v>
       </c>
       <c r="F28" s="18">
         <v>7.0601851851851847E-4</v>
@@ -1365,7 +1366,7 @@
         <v>51</v>
       </c>
       <c r="B29" s="7">
-        <v>27351</v>
+        <v>27356</v>
       </c>
       <c r="C29" s="12">
         <v>1.1574074074074073E-5</v>
@@ -1375,7 +1376,7 @@
       </c>
       <c r="E29" s="27">
         <f t="shared" si="0"/>
-        <v>1307529</v>
+        <v>1307524</v>
       </c>
       <c r="F29" s="18">
         <v>6.9444444444444444E-5</v>
@@ -1468,7 +1469,7 @@
     <row r="34" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B34" s="26">
         <f>SUM(B2:B33)</f>
-        <v>177477153</v>
+        <v>177477160</v>
       </c>
       <c r="D34" s="29">
         <f>SUM(D2:D33)</f>
@@ -1476,7 +1477,7 @@
       </c>
       <c r="E34" s="29">
         <f t="shared" si="0"/>
-        <v>1014298523989</v>
+        <v>1014298523982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>